<commit_message>
add google style docstring
</commit_message>
<xml_diff>
--- a/inputs/testcases.xlsx
+++ b/inputs/testcases.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,12 @@
       <b val="1"/>
       <color rgb="00006100"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00404040"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +74,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -83,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -93,6 +102,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -522,14 +532,14 @@
           <t>mindops-cmdb-skill</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "FAILED", "detail": "4 个字段中至少一个包含英文自然语言句子"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
+          <t>{"result": "PASS", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "PASS", "detail": "4 个字段全部中文合规"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
         </is>
       </c>
       <c r="F1" s="5" t="n"/>
@@ -559,7 +569,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "PASS", "detail": "4 个字段全部中文合规"}, "tool_choice": {"status": "FAILED", "detail": "期望工具未被调用: mindops-cmdb-skill"}}}</t>
+          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "FAILED", "detail": "4 个字段中至少一个包含英文自然语言句子"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
         </is>
       </c>
       <c r="F2" s="5" t="n"/>
@@ -612,14 +622,14 @@
           <t>mindops-cmdb-skill</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "FAILED", "detail": "4 个字段中至少一个包含英文自然语言句子"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
+          <t>{"result": "PASS", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "PASS", "detail": "4 个字段全部中文合规"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
         </is>
       </c>
       <c r="F4" s="5" t="n"/>
@@ -649,7 +659,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "PASS", "detail": "4 个字段全部中文合规"}, "tool_choice": {"status": "FAILED", "detail": "期望工具未被调用: mindops-cmdb-skill"}}}</t>
+          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "FAILED", "detail": "4 个字段中至少一个包含英文自然语言句子"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
         </is>
       </c>
       <c r="F5" s="5" t="n"/>
@@ -679,7 +689,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "FAILED", "detail": "4 个字段中至少一个包含英文自然语言句子"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
+          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "PASS", "detail": "4 个字段全部中文合规"}, "tool_choice": {"status": "FAILED", "detail": "期望工具未被调用: mindops-cmdb-skill"}}}</t>
         </is>
       </c>
       <c r="F6" s="5" t="n"/>
@@ -702,14 +712,14 @@
           <t>mindops-cmdb-skill</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "FAILED", "detail": "4 个字段中至少一个包含英文自然语言句子"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
+          <t>{"result": "PASS", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "PASS", "detail": "4 个字段全部中文合规"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
         </is>
       </c>
       <c r="F7" s="5" t="n"/>
@@ -739,7 +749,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "PASS", "detail": "4 个字段全部中文合规"}, "tool_choice": {"status": "FAILED", "detail": "期望工具未被调用: mindops-cmdb-skill"}}}</t>
+          <t>{"result": "FAILED", "checks": {"intent": {"status": "PASS", "detail": "意图: ASK"}, "i18n": {"status": "FAILED", "detail": "4 个字段中至少一个包含英文自然语言句子"}, "tool_choice": {"status": "PASS", "detail": "工具覆盖: mindops-cmdb-skill, 调用次数: 2"}}}</t>
         </is>
       </c>
       <c r="F8" s="5" t="n"/>

</xml_diff>